<commit_message>
feat: complete Apple/iPhone sub-brand fix, bracket promo filtering, and update all Google Sheets exports
</commit_message>
<xml_diff>
--- a/review/momo/Tickets & Services.xlsx
+++ b/review/momo/Tickets & Services.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">單品覆蓋!$A$1:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">審核!$A$1:$Y$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">審核!$A$1:$Z$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="N1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="236">
   <si>
     <t>【這個檔案怎麼用】</t>
   </si>
@@ -507,6 +507,12 @@
     <t>商品數</t>
   </si>
   <si>
+    <t>範例商品名稱</t>
+  </si>
+  <si>
+    <t>範例商品網址</t>
+  </si>
+  <si>
     <t>suggest brand name</t>
   </si>
   <si>
@@ -543,9 +549,6 @@
     <t>主要類目</t>
   </si>
   <si>
-    <t>範例商品名稱</t>
-  </si>
-  <si>
     <t>suggest brand id</t>
   </si>
   <si>
@@ -624,6 +627,48 @@
     <t>InfoThink</t>
   </si>
   <si>
+    <t>【懶散兔與啾先生】魔幻馬戲團雙層玻璃隨手瓶</t>
+  </si>
+  <si>
+    <t>【漢來海港餐廳】台北平日下午茶券4張(天母店)｜若完售請買15620140</t>
+  </si>
+  <si>
+    <t>【饗食天堂】新券!大組數超划算!平日晚餐/假日午餐通用券10張(TOP人氣吃到飽餐廳)</t>
+  </si>
+  <si>
+    <t>【Disney 迪士尼】怪獸電力公司-毛怪造型超柔擦手巾</t>
+  </si>
+  <si>
+    <t>【卡娜赫拉的小動物】浮雕造型醬料碟-P助款</t>
+  </si>
+  <si>
+    <t>【mofusand】日系清新感門簾-附伸縮桿</t>
+  </si>
+  <si>
+    <t>【跳跳虎】無線光學滑鼠</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/7632656</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/15266577</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/15266574</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/10255991</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/10640136</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/10128950</t>
+  </si>
+  <si>
+    <t>https://www.momoshop.com.tw/product/9587525</t>
+  </si>
+  <si>
     <t>HARBOUR 漢來海港餐廳</t>
   </si>
   <si>
@@ -709,27 +754,6 @@
   </si>
   <si>
     <t>Restaurant Voucher</t>
-  </si>
-  <si>
-    <t>【懶散兔與啾先生】魔幻馬戲團雙層玻璃隨手瓶</t>
-  </si>
-  <si>
-    <t>【漢來海港餐廳】台北平日下午茶券4張(天母店)｜若完售請買15620140</t>
-  </si>
-  <si>
-    <t>【饗食天堂】新券!大組數超划算!平日晚餐/假日午餐通用券10張(TOP人氣吃到飽餐廳)</t>
-  </si>
-  <si>
-    <t>【Disney 迪士尼】怪獸電力公司-毛怪造型超柔擦手巾</t>
-  </si>
-  <si>
-    <t>【卡娜赫拉的小動物】浮雕造型醬料碟-P助款</t>
-  </si>
-  <si>
-    <t>【mofusand】日系清新感門簾-附伸縮桿</t>
-  </si>
-  <si>
-    <t>【跳跳虎】無線光學滑鼠</t>
   </si>
   <si>
     <t>1083231</t>
@@ -1853,7 +1877,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y8"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="0" hidden="1" customWidth="1"/>
@@ -1863,19 +1887,20 @@
     <col min="6" max="6" width="7.7109375" customWidth="1"/>
     <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="7.7109375" customWidth="1"/>
-    <col min="9" max="9" width="24.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" customWidth="1"/>
-    <col min="11" max="13" width="26.7109375" customWidth="1"/>
-    <col min="14" max="17" width="22.7109375" customWidth="1"/>
-    <col min="18" max="18" width="45.7109375" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" customWidth="1"/>
-    <col min="20" max="20" width="16.7109375" customWidth="1"/>
-    <col min="21" max="21" width="40.7109375" customWidth="1"/>
-    <col min="22" max="24" width="22.7109375" customWidth="1"/>
-    <col min="25" max="25" width="18.7109375" customWidth="1"/>
+    <col min="9" max="9" width="40.7109375" customWidth="1"/>
+    <col min="10" max="10" width="36.7109375" customWidth="1"/>
+    <col min="11" max="11" width="24.7109375" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" customWidth="1"/>
+    <col min="13" max="15" width="26.7109375" customWidth="1"/>
+    <col min="16" max="19" width="22.7109375" customWidth="1"/>
+    <col min="20" max="20" width="45.7109375" customWidth="1"/>
+    <col min="21" max="21" width="18.7109375" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="23" max="25" width="22.7109375" customWidth="1"/>
+    <col min="26" max="26" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="32" customHeight="1">
+    <row r="1" spans="1:26" ht="32" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -1900,10 +1925,10 @@
       <c r="H1" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>144</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -1915,31 +1940,31 @@
       <c r="M1" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>149</v>
       </c>
       <c r="P1" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>154</v>
       </c>
       <c r="U1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>156</v>
       </c>
       <c r="W1" s="3" t="s">
@@ -1948,326 +1973,350 @@
       <c r="X1" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="3" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="2" spans="1:25">
+      <c r="Z1" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J2" t="s">
+        <v>190</v>
+      </c>
+      <c r="K2" t="s">
         <v>104</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>72</v>
       </c>
-      <c r="Q2" t="s">
-        <v>194</v>
-      </c>
-      <c r="R2" t="s">
-        <v>198</v>
-      </c>
       <c r="S2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="T2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="U2" t="s">
-        <v>211</v>
-      </c>
-      <c r="W2" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25">
+        <v>220</v>
+      </c>
+      <c r="V2" t="s">
+        <v>224</v>
+      </c>
+      <c r="X2" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H3">
         <v>19</v>
       </c>
       <c r="I3" t="s">
-        <v>182</v>
-      </c>
-      <c r="J3">
+        <v>184</v>
+      </c>
+      <c r="J3" t="s">
+        <v>191</v>
+      </c>
+      <c r="K3" t="s">
+        <v>197</v>
+      </c>
+      <c r="L3">
         <v>98</v>
       </c>
-      <c r="K3" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>195</v>
-      </c>
-      <c r="R3" t="s">
-        <v>199</v>
+      <c r="M3" t="s">
+        <v>201</v>
       </c>
       <c r="S3" t="s">
-        <v>178</v>
+        <v>210</v>
       </c>
       <c r="T3" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="U3" t="s">
-        <v>212</v>
+        <v>179</v>
       </c>
       <c r="V3" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25">
+        <v>225</v>
+      </c>
+      <c r="W3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H4">
         <v>8</v>
       </c>
       <c r="I4" t="s">
-        <v>179</v>
-      </c>
-      <c r="J4">
+        <v>185</v>
+      </c>
+      <c r="J4" t="s">
+        <v>192</v>
+      </c>
+      <c r="K4" t="s">
+        <v>180</v>
+      </c>
+      <c r="L4">
         <v>98</v>
       </c>
-      <c r="K4" t="s">
-        <v>187</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>195</v>
-      </c>
-      <c r="R4" t="s">
-        <v>200</v>
+      <c r="M4" t="s">
+        <v>202</v>
       </c>
       <c r="S4" t="s">
-        <v>179</v>
+        <v>210</v>
       </c>
       <c r="T4" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="U4" t="s">
-        <v>213</v>
+        <v>180</v>
       </c>
       <c r="V4" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25">
+        <v>225</v>
+      </c>
+      <c r="W4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H5">
         <v>6</v>
       </c>
       <c r="I5" t="s">
-        <v>183</v>
-      </c>
-      <c r="J5">
-        <v>85</v>
+        <v>186</v>
+      </c>
+      <c r="J5" t="s">
+        <v>193</v>
       </c>
       <c r="K5" t="s">
-        <v>188</v>
-      </c>
-      <c r="L5" t="s">
-        <v>192</v>
+        <v>198</v>
+      </c>
+      <c r="L5">
+        <v>83</v>
       </c>
       <c r="M5" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>196</v>
-      </c>
-      <c r="R5" t="s">
-        <v>201</v>
+        <v>203</v>
+      </c>
+      <c r="N5" t="s">
+        <v>207</v>
+      </c>
+      <c r="O5" t="s">
+        <v>208</v>
       </c>
       <c r="S5" t="s">
-        <v>180</v>
+        <v>211</v>
       </c>
       <c r="T5" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="U5" t="s">
-        <v>214</v>
+        <v>181</v>
       </c>
       <c r="V5" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25">
+        <v>224</v>
+      </c>
+      <c r="W5" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H6">
         <v>3</v>
       </c>
       <c r="I6" t="s">
-        <v>184</v>
-      </c>
-      <c r="J6">
-        <v>85</v>
+        <v>187</v>
+      </c>
+      <c r="J6" t="s">
+        <v>194</v>
       </c>
       <c r="K6" t="s">
-        <v>189</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>197</v>
-      </c>
-      <c r="R6" t="s">
-        <v>202</v>
+        <v>199</v>
+      </c>
+      <c r="L6">
+        <v>83</v>
+      </c>
+      <c r="M6" t="s">
+        <v>204</v>
       </c>
       <c r="S6" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="T6" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="U6" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="V6" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25">
+        <v>224</v>
+      </c>
+      <c r="W6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>185</v>
-      </c>
-      <c r="J7">
-        <v>85</v>
+        <v>188</v>
+      </c>
+      <c r="J7" t="s">
+        <v>195</v>
       </c>
       <c r="K7" t="s">
-        <v>190</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>197</v>
-      </c>
-      <c r="R7" t="s">
-        <v>203</v>
+        <v>200</v>
+      </c>
+      <c r="L7">
+        <v>83</v>
+      </c>
+      <c r="M7" t="s">
+        <v>205</v>
       </c>
       <c r="S7" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="T7" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="U7" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="V7" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25">
+        <v>224</v>
+      </c>
+      <c r="W7" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G8" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8" t="s">
-        <v>181</v>
-      </c>
-      <c r="J8">
-        <v>90</v>
+        <v>189</v>
+      </c>
+      <c r="J8" t="s">
+        <v>196</v>
       </c>
       <c r="K8" t="s">
-        <v>191</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>195</v>
-      </c>
-      <c r="R8" t="s">
-        <v>204</v>
+        <v>182</v>
+      </c>
+      <c r="L8">
+        <v>88</v>
+      </c>
+      <c r="M8" t="s">
+        <v>206</v>
       </c>
       <c r="S8" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="T8" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="U8" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="V8" t="s">
-        <v>223</v>
+        <v>224</v>
+      </c>
+      <c r="W8" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y8"/>
+  <autoFilter ref="A1:Z8"/>
   <conditionalFormatting sqref="B2:B8">
     <cfRule type="beginsWith" dxfId="3" priority="4" operator="beginsWith" text="①">
       <formula>LEFT(B2,1)="①"</formula>
@@ -2276,7 +2325,7 @@
       <formula>LEFT(B2,1)="④"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J8">
+  <conditionalFormatting sqref="L2:L8">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThanOrEqual">
       <formula>90</formula>
     </cfRule>
@@ -2288,26 +2337,26 @@
       <formula>75</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N8">
+  <conditionalFormatting sqref="P2:P8">
     <cfRule type="notContainsErrors" dxfId="5" priority="6">
-      <formula>NOT(ISERROR(N2))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O8">
-    <cfRule type="notContainsErrors" dxfId="5" priority="7">
-      <formula>NOT(ISERROR(O2))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P8">
-    <cfRule type="notContainsErrors" dxfId="5" priority="8">
       <formula>NOT(ISERROR(P2))</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q8">
+    <cfRule type="notContainsErrors" dxfId="5" priority="7">
+      <formula>NOT(ISERROR(Q2))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R8">
+    <cfRule type="notContainsErrors" dxfId="5" priority="8">
+      <formula>NOT(ISERROR(R2))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="填寫方式" prompt="v=同意｜1/2/3=選候選｜brand_id 或品牌名｜- =撤銷" sqref="N2:N8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="填寫方式" prompt="v=同意｜1/2/3=選候選｜brand_id 或品牌名｜- =撤銷" sqref="P2:P8">
       <formula1>"v,1,2,3,No brand,建議品牌庫新增品牌,-"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="O2:O8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="Q2:Q8">
       <formula1>"品牌欄與商品名稱皆無品牌,商品名稱【】為描述非品牌,相容/副廠配件,品牌欄標示無品牌,店家/賣場名稱非品牌,其他(請備註)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2332,31 +2381,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="32" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>141</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>